<commit_message>
Changing to master branch
New default branch
</commit_message>
<xml_diff>
--- a/SUEWSPrepare/Input/SUEWS_SiteSelect.xlsx
+++ b/SUEWSPrepare/Input/SUEWS_SiteSelect.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\xlinfr\Documents\PythonScripts\UMEP\SUEWSPrepare\Input\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="360" yWindow="345" windowWidth="18690" windowHeight="8835"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9336"/>
   </bookViews>
   <sheets>
     <sheet name="SUEWS_SiteSelect" sheetId="1" r:id="rId1"/>
@@ -13,12 +18,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Metadata!$H$1:$H$85</definedName>
   </definedNames>
-  <calcPr calcId="0" concurrentCalc="0"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="617" uniqueCount="247">
   <si>
     <t>Grid</t>
   </si>
@@ -741,13 +746,31 @@
   </si>
   <si>
     <t>old</t>
+  </si>
+  <si>
+    <t>TrafficRate_WD</t>
+  </si>
+  <si>
+    <t>TrafficRate_WE</t>
+  </si>
+  <si>
+    <t>IrrFr_Paved</t>
+  </si>
+  <si>
+    <t>IrrFr_Bldgs</t>
+  </si>
+  <si>
+    <t>IrrFr_BSoil</t>
+  </si>
+  <si>
+    <t>IrrFr_Water</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="18" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -882,6 +905,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="35">
@@ -1237,13 +1265,14 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1295,6 +1324,9 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
@@ -1342,7 +1374,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1377,7 +1409,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1586,112 +1618,116 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:CZ67"/>
-  <sheetFormatPr defaultColWidth="13.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:DD61"/>
+  <sheetFormatPr defaultColWidth="13.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="4.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="5" bestFit="1" customWidth="1"/>
     <col min="11" max="12" width="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="8" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="4" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="5" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="15" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="12" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="12" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="15" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="20" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="22" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="61" max="61" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="62" max="62" width="19" bestFit="1" customWidth="1"/>
-    <col min="63" max="63" width="12" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="19" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="12" bestFit="1" customWidth="1"/>
-    <col min="66" max="66" width="19" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="12" bestFit="1" customWidth="1"/>
-    <col min="68" max="68" width="19" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="12" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="19" bestFit="1" customWidth="1"/>
-    <col min="71" max="71" width="12" bestFit="1" customWidth="1"/>
-    <col min="72" max="72" width="19" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="12" bestFit="1" customWidth="1"/>
-    <col min="74" max="74" width="19" bestFit="1" customWidth="1"/>
-    <col min="75" max="75" width="12" bestFit="1" customWidth="1"/>
-    <col min="76" max="76" width="19" bestFit="1" customWidth="1"/>
-    <col min="77" max="77" width="12" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="21" bestFit="1" customWidth="1"/>
-    <col min="79" max="79" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="80" max="80" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="82" max="82" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="21" bestFit="1" customWidth="1"/>
-    <col min="85" max="85" width="9.140625" bestFit="1" customWidth="1"/>
-    <col min="86" max="88" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="89" max="91" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="92" max="96" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="97" max="101" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="102" max="102" width="1.7109375" bestFit="1" customWidth="1"/>
-    <col min="103" max="103" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="104" max="104" width="41.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="8" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="4" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="5" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="14.21875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="14" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="11" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="11" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="20.5546875" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="19.77734375" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="71" max="71" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="80" max="80" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="82" max="82" width="19" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="85" max="85" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="86" max="86" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="24.109375" bestFit="1" customWidth="1"/>
+    <col min="88" max="88" width="19.21875" bestFit="1" customWidth="1"/>
+    <col min="89" max="89" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="90" max="92" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="93" max="95" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="96" max="100" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="101" max="105" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="106" max="106" width="1.6640625" bestFit="1" customWidth="1"/>
+    <col min="107" max="107" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="108" max="108" width="38.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:104" x14ac:dyDescent="0.25">
-      <c r="A1" s="5">
+    <row r="1" spans="1:108" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="6">
         <v>1</v>
       </c>
-      <c r="B1" s="5">
+      <c r="B1" s="6">
         <v>2</v>
       </c>
-      <c r="C1" s="5">
+      <c r="C1" s="6">
         <v>3</v>
       </c>
-      <c r="D1" s="5">
+      <c r="D1" s="6">
         <v>4</v>
       </c>
       <c r="E1" s="5">
@@ -1700,7 +1736,7 @@
       <c r="F1" s="5">
         <v>6</v>
       </c>
-      <c r="G1" s="5">
+      <c r="G1" s="6">
         <v>7</v>
       </c>
       <c r="H1" s="5">
@@ -1985,1161 +2021,958 @@
       <c r="CW1" s="5">
         <v>101</v>
       </c>
-      <c r="CX1" s="5"/>
-      <c r="CY1" s="5"/>
-      <c r="CZ1" s="5"/>
-    </row>
-    <row r="2" spans="1:104" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="CX1" s="5">
+        <v>102</v>
+      </c>
+      <c r="CY1" s="5">
+        <v>103</v>
+      </c>
+      <c r="CZ1" s="5">
+        <v>104</v>
+      </c>
+      <c r="DA1" s="5">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:108" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" t="s">
         <v>235</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" t="s">
         <v>6</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" t="s">
         <v>7</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" t="s">
         <v>236</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" t="s">
         <v>8</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" t="s">
         <v>9</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="M2" t="s">
         <v>10</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="N2" t="s">
         <v>11</v>
       </c>
-      <c r="O2" s="5" t="s">
+      <c r="O2" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="5" t="s">
+      <c r="P2" t="s">
         <v>13</v>
       </c>
-      <c r="Q2" s="5" t="s">
+      <c r="Q2" t="s">
         <v>14</v>
       </c>
-      <c r="R2" s="5" t="s">
+      <c r="R2" t="s">
         <v>15</v>
       </c>
-      <c r="S2" s="5" t="s">
+      <c r="S2" t="s">
         <v>16</v>
       </c>
-      <c r="T2" s="5" t="s">
+      <c r="T2" t="s">
         <v>17</v>
       </c>
-      <c r="U2" s="5" t="s">
+      <c r="U2" t="s">
+        <v>243</v>
+      </c>
+      <c r="V2" t="s">
+        <v>244</v>
+      </c>
+      <c r="W2" t="s">
         <v>18</v>
       </c>
-      <c r="V2" s="5" t="s">
+      <c r="X2" t="s">
         <v>19</v>
       </c>
-      <c r="W2" s="5" t="s">
+      <c r="Y2" t="s">
         <v>20</v>
       </c>
-      <c r="X2" s="5" t="s">
+      <c r="Z2" t="s">
+        <v>245</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>246</v>
+      </c>
+      <c r="AB2" t="s">
         <v>21</v>
       </c>
-      <c r="Y2" s="5" t="s">
+      <c r="AC2" t="s">
         <v>22</v>
       </c>
-      <c r="Z2" s="5" t="s">
+      <c r="AD2" t="s">
         <v>23</v>
       </c>
-      <c r="AA2" s="5" t="s">
+      <c r="AE2" t="s">
         <v>24</v>
       </c>
-      <c r="AB2" s="5" t="s">
+      <c r="AF2" t="s">
         <v>25</v>
       </c>
-      <c r="AC2" s="5" t="s">
+      <c r="AG2" t="s">
         <v>26</v>
       </c>
-      <c r="AD2" s="5" t="s">
+      <c r="AH2" t="s">
         <v>27</v>
       </c>
-      <c r="AE2" s="5" t="s">
+      <c r="AI2" t="s">
         <v>28</v>
       </c>
-      <c r="AF2" s="5" t="s">
+      <c r="AJ2" t="s">
         <v>29</v>
       </c>
-      <c r="AG2" s="5" t="s">
+      <c r="AK2" t="s">
         <v>30</v>
       </c>
-      <c r="AH2" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="AI2" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="AJ2" s="5" t="s">
+      <c r="AL2" t="s">
+        <v>241</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>242</v>
+      </c>
+      <c r="AN2" t="s">
         <v>238</v>
       </c>
-      <c r="AK2" s="5" t="s">
+      <c r="AO2" t="s">
         <v>239</v>
       </c>
-      <c r="AL2" s="5" t="s">
+      <c r="AP2" t="s">
         <v>31</v>
       </c>
-      <c r="AM2" s="5" t="s">
+      <c r="AQ2" t="s">
         <v>32</v>
       </c>
-      <c r="AN2" s="5" t="s">
+      <c r="AR2" t="s">
         <v>33</v>
       </c>
-      <c r="AO2" s="5" t="s">
+      <c r="AS2" t="s">
         <v>34</v>
       </c>
-      <c r="AP2" s="5" t="s">
+      <c r="AT2" t="s">
         <v>35</v>
       </c>
-      <c r="AQ2" s="5" t="s">
+      <c r="AU2" t="s">
         <v>36</v>
       </c>
-      <c r="AR2" s="5" t="s">
+      <c r="AV2" t="s">
         <v>37</v>
       </c>
-      <c r="AS2" s="5" t="s">
+      <c r="AW2" t="s">
         <v>38</v>
       </c>
-      <c r="AT2" s="5" t="s">
+      <c r="AX2" t="s">
         <v>39</v>
       </c>
-      <c r="AU2" s="5" t="s">
+      <c r="AY2" t="s">
         <v>40</v>
       </c>
-      <c r="AV2" s="5" t="s">
+      <c r="AZ2" t="s">
         <v>41</v>
       </c>
-      <c r="AW2" s="5" t="s">
+      <c r="BA2" t="s">
         <v>42</v>
       </c>
-      <c r="AX2" s="5" t="s">
+      <c r="BB2" t="s">
         <v>43</v>
       </c>
-      <c r="AY2" s="5" t="s">
+      <c r="BC2" t="s">
         <v>44</v>
       </c>
-      <c r="AZ2" s="5" t="s">
+      <c r="BD2" t="s">
         <v>45</v>
       </c>
-      <c r="BA2" s="5" t="s">
+      <c r="BE2" t="s">
         <v>46</v>
       </c>
-      <c r="BB2" s="5" t="s">
+      <c r="BF2" t="s">
         <v>49</v>
       </c>
-      <c r="BC2" s="5" t="s">
+      <c r="BG2" t="s">
         <v>50</v>
       </c>
-      <c r="BD2" s="5" t="s">
+      <c r="BH2" t="s">
         <v>51</v>
       </c>
-      <c r="BE2" s="5" t="s">
+      <c r="BI2" t="s">
         <v>52</v>
       </c>
-      <c r="BF2" s="5" t="s">
+      <c r="BJ2" t="s">
         <v>53</v>
       </c>
-      <c r="BG2" s="5" t="s">
+      <c r="BK2" t="s">
         <v>54</v>
       </c>
-      <c r="BH2" s="5" t="s">
+      <c r="BL2" t="s">
         <v>55</v>
       </c>
-      <c r="BI2" s="5" t="s">
+      <c r="BM2" t="s">
         <v>56</v>
       </c>
-      <c r="BJ2" s="5" t="s">
+      <c r="BN2" t="s">
         <v>57</v>
       </c>
-      <c r="BK2" s="5" t="s">
+      <c r="BO2" t="s">
         <v>58</v>
       </c>
-      <c r="BL2" s="5" t="s">
+      <c r="BP2" t="s">
         <v>59</v>
       </c>
-      <c r="BM2" s="5" t="s">
+      <c r="BQ2" t="s">
         <v>60</v>
       </c>
-      <c r="BN2" s="5" t="s">
+      <c r="BR2" t="s">
         <v>61</v>
       </c>
-      <c r="BO2" s="5" t="s">
+      <c r="BS2" t="s">
         <v>62</v>
       </c>
-      <c r="BP2" s="5" t="s">
+      <c r="BT2" t="s">
         <v>63</v>
       </c>
-      <c r="BQ2" s="5" t="s">
+      <c r="BU2" t="s">
         <v>64</v>
       </c>
-      <c r="BR2" s="5" t="s">
+      <c r="BV2" t="s">
         <v>65</v>
       </c>
-      <c r="BS2" s="5" t="s">
+      <c r="BW2" t="s">
         <v>66</v>
       </c>
-      <c r="BT2" s="5" t="s">
+      <c r="BX2" t="s">
         <v>67</v>
       </c>
-      <c r="BU2" s="5" t="s">
+      <c r="BY2" t="s">
         <v>68</v>
       </c>
-      <c r="BV2" s="5" t="s">
+      <c r="BZ2" t="s">
         <v>69</v>
       </c>
-      <c r="BW2" s="5" t="s">
+      <c r="CA2" t="s">
         <v>70</v>
       </c>
-      <c r="BX2" s="5" t="s">
+      <c r="CB2" t="s">
         <v>71</v>
       </c>
-      <c r="BY2" s="5" t="s">
+      <c r="CC2" t="s">
         <v>72</v>
       </c>
-      <c r="BZ2" s="5" t="s">
+      <c r="CD2" t="s">
         <v>73</v>
       </c>
-      <c r="CA2" s="5" t="s">
+      <c r="CE2" t="s">
         <v>74</v>
       </c>
-      <c r="CB2" s="5" t="s">
+      <c r="CF2" t="s">
         <v>75</v>
       </c>
-      <c r="CC2" s="5" t="s">
+      <c r="CG2" t="s">
         <v>76</v>
       </c>
-      <c r="CD2" s="5" t="s">
+      <c r="CH2" t="s">
         <v>77</v>
       </c>
-      <c r="CE2" s="5" t="s">
+      <c r="CI2" t="s">
         <v>78</v>
       </c>
-      <c r="CF2" s="5" t="s">
+      <c r="CJ2" t="s">
         <v>79</v>
       </c>
-      <c r="CG2" s="5" t="s">
+      <c r="CK2" t="s">
         <v>214</v>
       </c>
-      <c r="CH2" s="5" t="s">
+      <c r="CL2" t="s">
         <v>215</v>
       </c>
-      <c r="CI2" s="5" t="s">
+      <c r="CM2" t="s">
         <v>216</v>
       </c>
-      <c r="CJ2" s="5" t="s">
+      <c r="CN2" t="s">
         <v>217</v>
       </c>
-      <c r="CK2" s="5" t="s">
+      <c r="CO2" t="s">
         <v>218</v>
       </c>
-      <c r="CL2" s="5" t="s">
+      <c r="CP2" t="s">
         <v>219</v>
       </c>
-      <c r="CM2" s="5" t="s">
+      <c r="CQ2" t="s">
         <v>220</v>
       </c>
-      <c r="CN2" s="5" t="s">
+      <c r="CR2" t="s">
         <v>221</v>
       </c>
-      <c r="CO2" s="5" t="s">
+      <c r="CS2" t="s">
         <v>222</v>
       </c>
-      <c r="CP2" s="5" t="s">
+      <c r="CT2" t="s">
         <v>223</v>
       </c>
-      <c r="CQ2" s="5" t="s">
+      <c r="CU2" t="s">
         <v>224</v>
       </c>
-      <c r="CR2" s="5" t="s">
+      <c r="CV2" t="s">
         <v>225</v>
       </c>
-      <c r="CS2" s="5" t="s">
+      <c r="CW2" t="s">
         <v>226</v>
       </c>
-      <c r="CT2" s="5" t="s">
+      <c r="CX2" t="s">
         <v>227</v>
       </c>
-      <c r="CU2" s="5" t="s">
+      <c r="CY2" t="s">
         <v>228</v>
       </c>
-      <c r="CV2" s="5" t="s">
+      <c r="CZ2" t="s">
         <v>229</v>
       </c>
-      <c r="CW2" s="5" t="s">
+      <c r="DA2" t="s">
         <v>230</v>
       </c>
-      <c r="CX2" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="CY2" s="5" t="s">
+      <c r="DB2" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="DC2" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="CZ2" s="5" t="s">
+      <c r="DD2" s="5" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="3" spans="1:104" x14ac:dyDescent="0.25">
-      <c r="A3" s="5">
-        <v>98</v>
-      </c>
-      <c r="B3" s="5">
-        <v>2012</v>
-      </c>
-      <c r="C3" s="5">
-        <v>85</v>
-      </c>
-      <c r="D3" s="5">
-        <v>302</v>
-      </c>
-      <c r="E3" s="5">
+    <row r="3" spans="1:108" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>2011</v>
+      </c>
+      <c r="C3">
+        <v>86</v>
+      </c>
+      <c r="D3">
+        <v>303</v>
+      </c>
+      <c r="E3">
         <v>51.51</v>
       </c>
-      <c r="F3" s="5">
-        <v>0.12</v>
-      </c>
-      <c r="G3" s="5">
+      <c r="F3">
+        <v>-0.12</v>
+      </c>
+      <c r="G3">
         <v>0</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3">
         <v>2221.56</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3">
         <v>10.7</v>
       </c>
-      <c r="J3" s="5">
+      <c r="J3">
         <v>49.6</v>
       </c>
-      <c r="K3" s="5">
+      <c r="K3">
         <v>1</v>
       </c>
-      <c r="L3" s="5">
+      <c r="L3">
         <v>0</v>
       </c>
-      <c r="M3" s="5">
+      <c r="M3">
         <v>0</v>
       </c>
-      <c r="N3" s="5">
+      <c r="N3">
         <v>0.43</v>
       </c>
-      <c r="O3" s="5">
+      <c r="O3">
         <v>0.38</v>
       </c>
-      <c r="P3" s="5">
+      <c r="P3">
         <v>0</v>
       </c>
-      <c r="Q3" s="5">
+      <c r="Q3">
         <v>0.02</v>
       </c>
-      <c r="R3" s="5">
+      <c r="R3">
         <v>0.03</v>
       </c>
-      <c r="S3" s="5">
+      <c r="S3">
         <v>0</v>
       </c>
-      <c r="T3" s="5">
+      <c r="T3">
         <v>0.14000000000000001</v>
       </c>
-      <c r="U3" s="5">
+      <c r="U3">
         <v>0</v>
       </c>
-      <c r="V3" s="5">
+      <c r="V3">
         <v>0</v>
       </c>
-      <c r="W3" s="5">
+      <c r="W3">
         <v>0</v>
       </c>
-      <c r="X3" s="5">
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
+        <v>0</v>
+      </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AB3">
         <v>22</v>
       </c>
-      <c r="Y3" s="5">
+      <c r="AC3">
         <v>13.1</v>
       </c>
-      <c r="Z3" s="5">
+      <c r="AD3">
         <v>13.1</v>
       </c>
-      <c r="AA3" s="5">
+      <c r="AE3">
         <v>1.9</v>
       </c>
-      <c r="AB3" s="5">
+      <c r="AF3">
         <v>14.2</v>
       </c>
-      <c r="AC3" s="5">
-        <v>-999</v>
-      </c>
-      <c r="AD3" s="5">
-        <v>-999</v>
-      </c>
-      <c r="AE3" s="5">
-        <v>-999</v>
-      </c>
-      <c r="AF3" s="5">
-        <v>-999</v>
-      </c>
-      <c r="AG3" s="5">
+      <c r="AG3">
+        <v>0.3</v>
+      </c>
+      <c r="AH3">
+        <v>0.3</v>
+      </c>
+      <c r="AI3">
+        <v>0.3</v>
+      </c>
+      <c r="AJ3">
         <v>204.58</v>
       </c>
-      <c r="AH3" s="5">
-        <v>-999</v>
-      </c>
-      <c r="AI3" s="5">
-        <v>-999</v>
-      </c>
-      <c r="AJ3" s="5">
+      <c r="AK3">
+        <v>204.58</v>
+      </c>
+      <c r="AL3">
+        <v>0.01</v>
+      </c>
+      <c r="AM3">
+        <v>0.01</v>
+      </c>
+      <c r="AN3">
         <v>0.88</v>
       </c>
-      <c r="AK3" s="5">
+      <c r="AO3">
         <v>0.88</v>
       </c>
-      <c r="AL3" s="5">
+      <c r="AP3">
         <v>661</v>
       </c>
-      <c r="AM3" s="5">
+      <c r="AQ3">
         <v>662</v>
       </c>
-      <c r="AN3" s="5">
+      <c r="AR3">
         <v>661</v>
       </c>
-      <c r="AO3" s="5">
+      <c r="AS3">
         <v>662</v>
       </c>
-      <c r="AP3" s="5">
+      <c r="AT3">
         <v>663</v>
       </c>
-      <c r="AQ3" s="5">
+      <c r="AU3">
         <v>663</v>
       </c>
-      <c r="AR3" s="5">
+      <c r="AV3">
         <v>661</v>
       </c>
-      <c r="AS3" s="5">
+      <c r="AW3">
         <v>0.25</v>
       </c>
-      <c r="AT3" s="5">
+      <c r="AX3">
         <v>1</v>
       </c>
-      <c r="AU3" s="5">
+      <c r="AY3">
         <v>10</v>
       </c>
-      <c r="AV3" s="5">
+      <c r="AZ3">
         <v>1</v>
       </c>
-      <c r="AW3" s="5">
+      <c r="BA3">
         <v>200</v>
       </c>
-      <c r="AX3" s="5">
-        <v>99999</v>
-      </c>
-      <c r="AY3" s="5">
-        <v>99999</v>
-      </c>
-      <c r="AZ3" s="5">
-        <v>99999</v>
-      </c>
-      <c r="BA3" s="5">
+      <c r="BB3">
+        <v>999</v>
+      </c>
+      <c r="BC3">
+        <v>999</v>
+      </c>
+      <c r="BD3">
+        <v>999</v>
+      </c>
+      <c r="BE3">
         <v>661</v>
       </c>
-      <c r="BB3" s="5">
-        <v>99999</v>
-      </c>
-      <c r="BC3" s="5">
-        <v>99999</v>
-      </c>
-      <c r="BD3" s="5">
-        <v>99999</v>
-      </c>
-      <c r="BE3" s="5">
-        <v>99999</v>
-      </c>
-      <c r="BF3" s="5">
-        <v>99999</v>
-      </c>
-      <c r="BG3" s="5">
+      <c r="BF3">
+        <v>999</v>
+      </c>
+      <c r="BG3">
+        <v>999</v>
+      </c>
+      <c r="BH3">
+        <v>999</v>
+      </c>
+      <c r="BI3">
+        <v>999</v>
+      </c>
+      <c r="BJ3">
+        <v>999</v>
+      </c>
+      <c r="BK3">
         <v>0</v>
       </c>
-      <c r="BH3" s="5">
+      <c r="BL3">
         <v>0</v>
       </c>
-      <c r="BI3" s="5">
+      <c r="BM3">
         <v>100</v>
       </c>
-      <c r="BJ3" s="5">
+      <c r="BN3">
         <v>0</v>
       </c>
-      <c r="BK3" s="5">
+      <c r="BO3">
         <v>0</v>
       </c>
-      <c r="BL3" s="5">
+      <c r="BP3">
         <v>0</v>
       </c>
-      <c r="BM3" s="5">
+      <c r="BQ3">
         <v>0</v>
       </c>
-      <c r="BN3" s="5">
+      <c r="BR3">
         <v>0</v>
       </c>
-      <c r="BO3" s="5">
+      <c r="BS3">
         <v>0</v>
       </c>
-      <c r="BP3" s="5">
+      <c r="BT3">
         <v>0</v>
       </c>
-      <c r="BQ3" s="5">
+      <c r="BU3">
         <v>0</v>
       </c>
-      <c r="BR3" s="5">
+      <c r="BV3">
         <v>0</v>
       </c>
-      <c r="BS3" s="5">
+      <c r="BW3">
         <v>0</v>
       </c>
-      <c r="BT3" s="5">
+      <c r="BX3">
         <v>0</v>
       </c>
-      <c r="BU3" s="5">
+      <c r="BY3">
         <v>0</v>
       </c>
-      <c r="BV3" s="5">
+      <c r="BZ3">
         <v>0</v>
       </c>
-      <c r="BW3" s="5">
+      <c r="CA3">
         <v>0</v>
       </c>
-      <c r="BX3" s="5">
+      <c r="CB3">
         <v>0</v>
       </c>
-      <c r="BY3" s="5">
+      <c r="CC3">
         <v>0</v>
       </c>
-      <c r="BZ3" s="5">
+      <c r="CD3">
         <v>661</v>
       </c>
-      <c r="CA3" s="5">
+      <c r="CE3">
         <v>662</v>
       </c>
-      <c r="CB3" s="5">
+      <c r="CF3">
         <v>663</v>
       </c>
-      <c r="CC3" s="5">
+      <c r="CG3">
         <v>664</v>
       </c>
-      <c r="CD3" s="5">
+      <c r="CH3">
         <v>665</v>
       </c>
-      <c r="CE3" s="5">
+      <c r="CI3">
         <v>666</v>
       </c>
-      <c r="CF3" s="5">
+      <c r="CJ3">
         <v>667</v>
       </c>
-      <c r="CG3" s="5">
-        <v>1.08</v>
-      </c>
-      <c r="CH3" s="5">
-        <v>0.15</v>
-      </c>
-      <c r="CI3" s="5">
-        <v>0.05</v>
-      </c>
-      <c r="CJ3" s="5">
-        <v>0.8</v>
-      </c>
-      <c r="CK3" s="5">
+      <c r="CK3">
+        <v>7000</v>
+      </c>
+      <c r="CL3">
+        <v>0</v>
+      </c>
+      <c r="CM3">
+        <v>1</v>
+      </c>
+      <c r="CN3">
+        <v>0</v>
+      </c>
+      <c r="CO3">
         <v>806</v>
       </c>
-      <c r="CL3" s="5">
+      <c r="CP3">
         <v>807</v>
       </c>
-      <c r="CM3" s="5">
+      <c r="CQ3">
         <v>808</v>
       </c>
-      <c r="CN3" s="5">
-        <v>0.15</v>
-      </c>
-      <c r="CO3" s="5">
-        <v>0.45</v>
-      </c>
-      <c r="CP3" s="5">
-        <v>0.05</v>
-      </c>
-      <c r="CQ3" s="5">
-        <v>0.1</v>
-      </c>
-      <c r="CR3" s="5">
-        <v>0.25</v>
-      </c>
-      <c r="CS3" s="5">
+      <c r="CR3">
+        <v>1</v>
+      </c>
+      <c r="CS3">
+        <v>0</v>
+      </c>
+      <c r="CT3">
+        <v>0</v>
+      </c>
+      <c r="CU3">
+        <v>0</v>
+      </c>
+      <c r="CV3">
+        <v>0</v>
+      </c>
+      <c r="CW3">
         <v>801</v>
       </c>
-      <c r="CT3" s="5">
-        <v>8021</v>
-      </c>
-      <c r="CU3" s="5">
-        <v>8022</v>
-      </c>
-      <c r="CV3" s="5">
+      <c r="CX3">
+        <v>802</v>
+      </c>
+      <c r="CY3">
         <v>803</v>
       </c>
-      <c r="CW3" s="5">
-        <v>8041</v>
-      </c>
-      <c r="CX3" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="CY3" s="5" t="s">
+      <c r="CZ3">
+        <v>804</v>
+      </c>
+      <c r="DA3">
+        <v>805</v>
+      </c>
+      <c r="DB3" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="DC3" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="CZ3" s="5" t="s">
+      <c r="DD3" s="5" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="4" spans="1:104" x14ac:dyDescent="0.25">
-      <c r="A4" s="5">
+    <row r="4" spans="1:108" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>-9</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
-      <c r="M4" s="5"/>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-      <c r="R4" s="5"/>
-      <c r="S4" s="5"/>
-      <c r="T4" s="5"/>
-      <c r="U4" s="5"/>
-      <c r="V4" s="5"/>
-      <c r="W4" s="5"/>
-      <c r="X4" s="5"/>
-      <c r="Y4" s="5"/>
-      <c r="Z4" s="5"/>
-      <c r="AA4" s="5"/>
-      <c r="AB4" s="5"/>
-      <c r="AC4" s="5"/>
-      <c r="AD4" s="5"/>
-      <c r="AE4" s="5"/>
-      <c r="AF4" s="5"/>
-      <c r="AG4" s="5"/>
-      <c r="AH4" s="5"/>
-      <c r="AI4" s="5"/>
-      <c r="AJ4" s="5"/>
-      <c r="AK4" s="5"/>
-      <c r="AL4" s="5"/>
-      <c r="AM4" s="5"/>
-      <c r="AN4" s="5"/>
-      <c r="AO4" s="5"/>
-      <c r="AP4" s="5"/>
-      <c r="AQ4" s="5"/>
-      <c r="AR4" s="5"/>
-      <c r="AS4" s="5"/>
-      <c r="AT4" s="5"/>
-      <c r="AU4" s="5"/>
-      <c r="AV4" s="5"/>
-      <c r="AW4" s="5"/>
-      <c r="AX4" s="5"/>
-      <c r="AY4" s="5"/>
-      <c r="AZ4" s="5"/>
-      <c r="BA4" s="5"/>
-      <c r="BB4" s="5"/>
-      <c r="BC4" s="5"/>
-      <c r="BD4" s="5"/>
-      <c r="BE4" s="5"/>
-      <c r="BF4" s="5"/>
-      <c r="BG4" s="5"/>
-      <c r="BH4" s="5"/>
-      <c r="BI4" s="5"/>
-      <c r="BJ4" s="5"/>
-      <c r="BK4" s="5"/>
-      <c r="BL4" s="5"/>
-      <c r="BM4" s="5"/>
-      <c r="BN4" s="5"/>
-      <c r="BO4" s="5"/>
-      <c r="BP4" s="5"/>
-      <c r="BQ4" s="5"/>
-      <c r="BR4" s="5"/>
-      <c r="BS4" s="5"/>
-      <c r="BT4" s="5"/>
-      <c r="BU4" s="5"/>
-      <c r="BV4" s="5"/>
-      <c r="BW4" s="5"/>
-      <c r="BX4" s="5"/>
-      <c r="BY4" s="5"/>
-      <c r="BZ4" s="5"/>
-      <c r="CA4" s="5"/>
-      <c r="CB4" s="5"/>
-      <c r="CC4" s="5"/>
-      <c r="CD4" s="5"/>
-      <c r="CE4" s="5"/>
-      <c r="CF4" s="5"/>
-      <c r="CG4" s="5"/>
-      <c r="CH4" s="5"/>
-      <c r="CI4" s="5"/>
-      <c r="CJ4" s="5"/>
-      <c r="CK4" s="5"/>
-      <c r="CL4" s="5"/>
-      <c r="CM4" s="5"/>
-      <c r="CN4" s="5"/>
-      <c r="CO4" s="5"/>
-      <c r="CP4" s="5"/>
-      <c r="CQ4" s="5"/>
-      <c r="CR4" s="5"/>
-      <c r="CS4" s="5"/>
-      <c r="CT4" s="5"/>
-      <c r="CU4" s="5"/>
-      <c r="CV4" s="5"/>
-      <c r="CW4" s="5"/>
-      <c r="CX4" s="5"/>
-      <c r="CY4" s="5"/>
-      <c r="CZ4" s="5"/>
-    </row>
-    <row r="5" spans="1:104" x14ac:dyDescent="0.25">
-      <c r="A5" s="5">
+    </row>
+    <row r="5" spans="1:108" x14ac:dyDescent="0.3">
+      <c r="A5">
         <v>-9</v>
       </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-      <c r="M5" s="5"/>
-      <c r="N5" s="5"/>
-      <c r="O5" s="5"/>
-      <c r="P5" s="5"/>
-      <c r="Q5" s="5"/>
-      <c r="R5" s="5"/>
-      <c r="S5" s="5"/>
-      <c r="T5" s="5"/>
-      <c r="U5" s="5"/>
-      <c r="V5" s="5"/>
-      <c r="W5" s="5"/>
-      <c r="X5" s="5"/>
-      <c r="Y5" s="5"/>
-      <c r="Z5" s="5"/>
-      <c r="AA5" s="5"/>
-      <c r="AB5" s="5"/>
-      <c r="AC5" s="5"/>
-      <c r="AD5" s="5"/>
-      <c r="AE5" s="5"/>
-      <c r="AF5" s="5"/>
-      <c r="AG5" s="5"/>
-      <c r="AH5" s="5"/>
-      <c r="AI5" s="5"/>
-      <c r="AJ5" s="5"/>
-      <c r="AK5" s="5"/>
-      <c r="AL5" s="5"/>
-      <c r="AM5" s="5"/>
-      <c r="AN5" s="5"/>
-      <c r="AO5" s="5"/>
-      <c r="AP5" s="5"/>
-      <c r="AQ5" s="5"/>
-      <c r="AR5" s="5"/>
-      <c r="AS5" s="5"/>
-      <c r="AT5" s="5"/>
-      <c r="AU5" s="5"/>
-      <c r="AV5" s="5"/>
-      <c r="AW5" s="5"/>
-      <c r="AX5" s="5"/>
-      <c r="AY5" s="5"/>
-      <c r="AZ5" s="5"/>
-      <c r="BA5" s="5"/>
-      <c r="BB5" s="5"/>
-      <c r="BC5" s="5"/>
-      <c r="BD5" s="5"/>
-      <c r="BE5" s="5"/>
-      <c r="BF5" s="5"/>
-      <c r="BG5" s="5"/>
-      <c r="BH5" s="5"/>
-      <c r="BI5" s="5"/>
-      <c r="BJ5" s="5"/>
-      <c r="BK5" s="5"/>
-      <c r="BL5" s="5"/>
-      <c r="BM5" s="5"/>
-      <c r="BN5" s="5"/>
-      <c r="BO5" s="5"/>
-      <c r="BP5" s="5"/>
-      <c r="BQ5" s="5"/>
-      <c r="BR5" s="5"/>
-      <c r="BS5" s="5"/>
-      <c r="BT5" s="5"/>
-      <c r="BU5" s="5"/>
-      <c r="BV5" s="5"/>
-      <c r="BW5" s="5"/>
-      <c r="BX5" s="5"/>
-      <c r="BY5" s="5"/>
-      <c r="BZ5" s="5"/>
-      <c r="CA5" s="5"/>
-      <c r="CB5" s="5"/>
-      <c r="CC5" s="5"/>
-      <c r="CD5" s="5"/>
-      <c r="CE5" s="5"/>
-      <c r="CF5" s="5"/>
-      <c r="CG5" s="5"/>
-      <c r="CH5" s="5"/>
-      <c r="CI5" s="5"/>
-      <c r="CJ5" s="5"/>
-      <c r="CK5" s="5"/>
-      <c r="CL5" s="5"/>
-      <c r="CM5" s="5"/>
-      <c r="CN5" s="5"/>
-      <c r="CO5" s="5"/>
-      <c r="CP5" s="5"/>
-      <c r="CQ5" s="5"/>
-      <c r="CR5" s="5"/>
-      <c r="CS5" s="5"/>
-      <c r="CT5" s="5"/>
-      <c r="CU5" s="5"/>
-      <c r="CV5" s="5"/>
-      <c r="CW5" s="5"/>
-      <c r="CX5" s="5"/>
-      <c r="CY5" s="5"/>
-      <c r="CZ5" s="5"/>
-    </row>
-    <row r="6" spans="1:104" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:104" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:104" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="1:104" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:104" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="11" spans="1:104" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="12" spans="1:104" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="13" spans="1:104" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="14" spans="1:104" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:104" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="16" spans="1:104" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:108" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
         <v>80</v>
       </c>
     </row>
@@ -3152,20 +2985,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I106"/>
-  <sheetFormatPr defaultColWidth="54" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="54" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" customWidth="1"/>
-    <col min="5" max="5" width="26.140625" customWidth="1"/>
-    <col min="6" max="6" width="33.85546875" customWidth="1"/>
-    <col min="7" max="7" width="20.85546875" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" customWidth="1"/>
-    <col min="9" max="9" width="21.28515625" customWidth="1"/>
-    <col min="10" max="40" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.33203125" customWidth="1"/>
+    <col min="4" max="4" width="19.88671875" customWidth="1"/>
+    <col min="5" max="5" width="26.109375" customWidth="1"/>
+    <col min="6" max="6" width="33.88671875" customWidth="1"/>
+    <col min="7" max="7" width="20.88671875" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" customWidth="1"/>
+    <col min="9" max="9" width="21.33203125" customWidth="1"/>
+    <col min="10" max="40" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>200</v>
       </c>
@@ -3191,7 +3024,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3217,7 +3050,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3240,7 +3073,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -3263,7 +3096,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -3286,7 +3119,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3312,7 +3145,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3338,7 +3171,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3353,7 +3186,7 @@
       <c r="H8" s="2"/>
       <c r="I8" s="5"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3379,7 +3212,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3405,7 +3238,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3420,7 +3253,7 @@
       <c r="H11" s="3"/>
       <c r="I11" s="5"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3444,7 +3277,7 @@
       </c>
       <c r="H12" s="3"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3465,7 +3298,7 @@
       </c>
       <c r="H13" s="3"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3486,7 +3319,7 @@
       </c>
       <c r="H14" s="3"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3506,7 +3339,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3526,7 +3359,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3546,7 +3379,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3566,7 +3399,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3586,7 +3419,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -3606,7 +3439,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -3626,7 +3459,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -3644,7 +3477,7 @@
       </c>
       <c r="H22" s="3"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -3662,7 +3495,7 @@
       </c>
       <c r="H23" s="3"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -3680,7 +3513,7 @@
       </c>
       <c r="H24" s="3"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -3703,7 +3536,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -3726,7 +3559,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -3749,7 +3582,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -3773,7 +3606,7 @@
       </c>
       <c r="H28" s="3"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -3797,7 +3630,7 @@
       </c>
       <c r="H29" s="3"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -3817,7 +3650,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3837,7 +3670,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -3857,7 +3690,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -3880,7 +3713,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3903,7 +3736,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3914,7 +3747,7 @@
       <c r="G35" s="5"/>
       <c r="H35" s="3"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3928,7 +3761,7 @@
       <c r="G36" s="5"/>
       <c r="H36" s="3"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3942,7 +3775,7 @@
       <c r="G37" s="5"/>
       <c r="H37" s="3"/>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3956,7 +3789,7 @@
       <c r="G38" s="5"/>
       <c r="H38" s="3"/>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3979,7 +3812,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -4002,7 +3835,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>40</v>
       </c>
@@ -4025,7 +3858,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -4048,7 +3881,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -4071,7 +3904,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -4094,7 +3927,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -4117,7 +3950,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -4138,7 +3971,7 @@
       </c>
       <c r="H46" s="3"/>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -4159,7 +3992,7 @@
       </c>
       <c r="H47" s="3"/>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -4180,7 +4013,7 @@
       </c>
       <c r="H48" s="3"/>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -4198,7 +4031,7 @@
       </c>
       <c r="H49" s="3"/>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -4221,7 +4054,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -4244,7 +4077,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -4267,7 +4100,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -4290,7 +4123,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -4313,7 +4146,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -4333,7 +4166,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>55</v>
       </c>
@@ -4356,7 +4189,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -4379,7 +4212,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -4402,7 +4235,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
@@ -4425,7 +4258,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>59</v>
       </c>
@@ -4446,7 +4279,7 @@
       </c>
       <c r="H60" s="3"/>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>60</v>
       </c>
@@ -4464,7 +4297,7 @@
       </c>
       <c r="H61" s="3"/>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>61</v>
       </c>
@@ -4485,7 +4318,7 @@
       </c>
       <c r="H62" s="3"/>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>62</v>
       </c>
@@ -4503,7 +4336,7 @@
       </c>
       <c r="H63" s="3"/>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>63</v>
       </c>
@@ -4521,7 +4354,7 @@
       </c>
       <c r="H64" s="3"/>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>64</v>
       </c>
@@ -4539,7 +4372,7 @@
       </c>
       <c r="H65" s="3"/>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>65</v>
       </c>
@@ -4557,7 +4390,7 @@
       </c>
       <c r="H66" s="3"/>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>66</v>
       </c>
@@ -4575,7 +4408,7 @@
       </c>
       <c r="H67" s="3"/>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>67</v>
       </c>
@@ -4593,7 +4426,7 @@
       </c>
       <c r="H68" s="3"/>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>68</v>
       </c>
@@ -4611,7 +4444,7 @@
       </c>
       <c r="H69" s="3"/>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>69</v>
       </c>
@@ -4629,7 +4462,7 @@
       </c>
       <c r="H70" s="3"/>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>70</v>
       </c>
@@ -4647,7 +4480,7 @@
       </c>
       <c r="H71" s="3"/>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>71</v>
       </c>
@@ -4665,7 +4498,7 @@
       </c>
       <c r="H72" s="3"/>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>72</v>
       </c>
@@ -4683,7 +4516,7 @@
       </c>
       <c r="H73" s="3"/>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>73</v>
       </c>
@@ -4701,7 +4534,7 @@
       </c>
       <c r="H74" s="3"/>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
         <v>74</v>
       </c>
@@ -4719,7 +4552,7 @@
       </c>
       <c r="H75" s="3"/>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
         <v>75</v>
       </c>
@@ -4737,7 +4570,7 @@
       </c>
       <c r="H76" s="3"/>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="2">
         <v>76</v>
       </c>
@@ -4755,7 +4588,7 @@
       </c>
       <c r="H77" s="3"/>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -4773,7 +4606,7 @@
       </c>
       <c r="H78" s="3"/>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -4793,7 +4626,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -4813,7 +4646,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -4833,7 +4666,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -4853,7 +4686,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
         <v>82</v>
       </c>
@@ -4873,7 +4706,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -4893,7 +4726,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -4913,7 +4746,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -4921,7 +4754,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -4929,7 +4762,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -4937,7 +4770,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -4950,7 +4783,7 @@
       <c r="G89" s="5"/>
       <c r="H89" s="5"/>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -4963,7 +4796,7 @@
       <c r="G90" s="5"/>
       <c r="H90" s="5"/>
     </row>
-    <row r="91" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -4971,7 +4804,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="92" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -4979,7 +4812,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="93" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -4987,7 +4820,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="94" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -4995,7 +4828,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="95" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -5003,7 +4836,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="96" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -5011,7 +4844,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="97" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -5019,7 +4852,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="98" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -5027,7 +4860,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="99" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -5035,7 +4868,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="100" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2">
         <v>99</v>
       </c>
@@ -5043,7 +4876,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="101" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -5056,7 +4889,7 @@
       <c r="G101"/>
       <c r="H101"/>
     </row>
-    <row r="102" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A102" s="2">
         <v>101</v>
       </c>
@@ -5069,12 +4902,12 @@
       <c r="G102"/>
       <c r="H102"/>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>54</v>
       </c>
@@ -5097,7 +4930,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>55</v>
       </c>

</xml_diff>